<commit_message>
feat(data): 100+ turk tarifi seed verisi ve kalori hesaplama betikleri
</commit_message>
<xml_diff>
--- a/docs/Kalori_Sayaci_20_Gunluk_Staj_Plani.xlsx
+++ b/docs/Kalori_Sayaci_20_Gunluk_Staj_Plani.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekin\Desktop\FDN\kalori\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30C622A9-FAD5-496E-8881-9D02168DAF46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D6C0B0-779C-4B1F-8580-E7A5AD27B55C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ozet Dashboard" sheetId="1" r:id="rId1"/>
@@ -3270,30 +3270,30 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3715,7 +3715,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="32"/>
@@ -3725,7 +3725,7 @@
       <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="34" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="32"/>
@@ -3743,169 +3743,169 @@
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
     </row>
     <row r="6" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="34"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="39"/>
     </row>
     <row r="7" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="34"/>
-      <c r="F7" s="34"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
     </row>
     <row r="8" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
     </row>
     <row r="9" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
     </row>
     <row r="10" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
     </row>
     <row r="11" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
     </row>
     <row r="12" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="34"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="39"/>
     </row>
     <row r="13" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
     </row>
     <row r="14" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="33" t="s">
+      <c r="B14" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="34"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="39"/>
     </row>
     <row r="15" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="33" t="s">
+      <c r="B15" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
     </row>
     <row r="16" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="33" t="s">
+      <c r="B16" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="39"/>
+      <c r="F16" s="39"/>
     </row>
     <row r="17" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="33" t="s">
+      <c r="B17" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="34"/>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="39"/>
+      <c r="F17" s="39"/>
     </row>
     <row r="18" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="33" t="s">
+      <c r="B18" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="34"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="39"/>
+      <c r="F18" s="39"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
@@ -3946,11 +3946,11 @@
       </c>
       <c r="D22" s="6">
         <f>SUMIFS('Sprint Plani'!$H$4:$H$77,'Sprint Plani'!$A$4:$A$77,$A22,'Sprint Plani'!$K$4:$K$77,"Tamamlandı")</f>
-        <v>8.5</v>
+        <v>15</v>
       </c>
       <c r="E22" s="7">
         <f>IFERROR($D22/$C22,0)</f>
-        <v>0.20238095238095238</v>
+        <v>0.35714285714285715</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>39</v>
@@ -4042,11 +4042,11 @@
       </c>
       <c r="D26" s="10">
         <f>SUM(D22:D25)</f>
-        <v>8.5</v>
+        <v>15</v>
       </c>
       <c r="E26" s="11">
         <f>IFERROR(D26/C26,0)</f>
-        <v>5.1051051051051052E-2</v>
+        <v>9.0090090090090086E-2</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>47</v>
@@ -4084,11 +4084,11 @@
       </c>
       <c r="C30" s="14">
         <f>COUNTIF('Sprint Plani'!$K$4:$K$77,$B30)</f>
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D30" s="15">
         <f>SUMIF('Sprint Plani'!$K$4:$K$77,$B30,'Sprint Plani'!$H$4:$H$77)</f>
-        <v>158</v>
+        <v>151.5</v>
       </c>
       <c r="E30" s="14"/>
       <c r="F30" s="16" t="s">
@@ -4124,11 +4124,11 @@
       </c>
       <c r="C32" s="14">
         <f>COUNTIF('Sprint Plani'!$K$4:$K$77,$B32)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D32" s="15">
         <f>SUMIF('Sprint Plani'!$K$4:$K$77,$B32,'Sprint Plani'!$H$4:$H$77)</f>
-        <v>8.5</v>
+        <v>15</v>
       </c>
       <c r="E32" s="14"/>
       <c r="F32" s="16" t="s">
@@ -4241,7 +4241,7 @@
       </c>
     </row>
     <row r="40" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="31" t="s">
+      <c r="A40" s="40" t="s">
         <v>73</v>
       </c>
       <c r="B40" s="32"/>
@@ -4251,7 +4251,7 @@
       <c r="F40" s="32"/>
     </row>
     <row r="41" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="31" t="s">
+      <c r="A41" s="40" t="s">
         <v>74</v>
       </c>
       <c r="B41" s="32"/>
@@ -4261,7 +4261,7 @@
       <c r="F41" s="32"/>
     </row>
     <row r="42" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="31" t="s">
+      <c r="A42" s="40" t="s">
         <v>75</v>
       </c>
       <c r="B42" s="32"/>
@@ -4271,7 +4271,7 @@
       <c r="F42" s="32"/>
     </row>
     <row r="43" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="31" t="s">
+      <c r="A43" s="40" t="s">
         <v>76</v>
       </c>
       <c r="B43" s="32"/>
@@ -4281,7 +4281,7 @@
       <c r="F43" s="32"/>
     </row>
     <row r="44" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="31" t="s">
+      <c r="A44" s="40" t="s">
         <v>77</v>
       </c>
       <c r="B44" s="32"/>
@@ -4296,7 +4296,7 @@
       </c>
     </row>
     <row r="47" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="35" t="s">
+      <c r="A47" s="37" t="s">
         <v>79</v>
       </c>
       <c r="B47" s="32"/>
@@ -4306,7 +4306,7 @@
       <c r="F47" s="32"/>
     </row>
     <row r="48" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="35" t="s">
+      <c r="A48" s="37" t="s">
         <v>80</v>
       </c>
       <c r="B48" s="32"/>
@@ -4316,7 +4316,7 @@
       <c r="F48" s="32"/>
     </row>
     <row r="49" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="35" t="s">
+      <c r="A49" s="37" t="s">
         <v>81</v>
       </c>
       <c r="B49" s="32"/>
@@ -4326,7 +4326,7 @@
       <c r="F49" s="32"/>
     </row>
     <row r="50" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="35" t="s">
+      <c r="A50" s="37" t="s">
         <v>82</v>
       </c>
       <c r="B50" s="32"/>
@@ -4336,7 +4336,7 @@
       <c r="F50" s="32"/>
     </row>
     <row r="51" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="35" t="s">
+      <c r="A51" s="37" t="s">
         <v>83</v>
       </c>
       <c r="B51" s="32"/>
@@ -4347,6 +4347,16 @@
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B16:F16"/>
     <mergeCell ref="A51:F51"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B15:F15"/>
@@ -4363,16 +4373,6 @@
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="A43:F43"/>
     <mergeCell ref="A44:F44"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="A40:F40"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="A41:F41"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="A48:F48"/>
-    <mergeCell ref="A49:F49"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4399,7 +4399,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="31" t="s">
         <v>84</v>
       </c>
       <c r="B1" s="32"/>
@@ -4414,7 +4414,7 @@
       <c r="K1" s="32"/>
     </row>
     <row r="2" spans="1:11" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="34" t="s">
         <v>85</v>
       </c>
       <c r="B2" s="32"/>
@@ -4635,7 +4635,7 @@
         <v>110</v>
       </c>
       <c r="K8" s="17" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="41.85" customHeight="1" x14ac:dyDescent="0.3">
@@ -4670,7 +4670,7 @@
         <v>116</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="41.85" customHeight="1" x14ac:dyDescent="0.3">
@@ -4705,7 +4705,7 @@
         <v>116</v>
       </c>
       <c r="K10" s="17" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="41.85" customHeight="1" x14ac:dyDescent="0.3">
@@ -7054,15 +7054,15 @@
       </c>
     </row>
     <row r="78" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="39" t="s">
+      <c r="A78" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="B78" s="40"/>
-      <c r="C78" s="40"/>
-      <c r="D78" s="40"/>
-      <c r="E78" s="40"/>
-      <c r="F78" s="40"/>
-      <c r="G78" s="40"/>
+      <c r="B78" s="36"/>
+      <c r="C78" s="36"/>
+      <c r="D78" s="36"/>
+      <c r="E78" s="36"/>
+      <c r="F78" s="36"/>
+      <c r="G78" s="36"/>
       <c r="H78" s="24">
         <f>SUM(H4:H77)</f>
         <v>166.5</v>
@@ -7075,7 +7075,7 @@
       <c r="K78" s="23"/>
     </row>
     <row r="80" spans="1:11" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="38" t="s">
+      <c r="A80" s="33" t="s">
         <v>454</v>
       </c>
       <c r="B80" s="32"/>
@@ -7090,7 +7090,7 @@
       <c r="K80" s="32"/>
     </row>
     <row r="81" spans="1:11" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="38" t="s">
+      <c r="A81" s="33" t="s">
         <v>455</v>
       </c>
       <c r="B81" s="32"/>
@@ -7105,7 +7105,7 @@
       <c r="K81" s="32"/>
     </row>
     <row r="82" spans="1:11" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="38" t="s">
+      <c r="A82" s="33" t="s">
         <v>456</v>
       </c>
       <c r="B82" s="32"/>
@@ -7177,7 +7177,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="31" t="s">
         <v>457</v>
       </c>
       <c r="B1" s="32"/>
@@ -7189,7 +7189,7 @@
       <c r="H1" s="32"/>
     </row>
     <row r="2" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="34" t="s">
         <v>458</v>
       </c>
       <c r="B2" s="32"/>
@@ -7695,7 +7695,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="31" t="s">
         <v>549</v>
       </c>
       <c r="B1" s="32"/>
@@ -7706,7 +7706,7 @@
       <c r="G1" s="32"/>
     </row>
     <row r="2" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="34" t="s">
         <v>550</v>
       </c>
       <c r="B2" s="32"/>
@@ -8067,10 +8067,10 @@
       <c r="C19" s="41" t="s">
         <v>602</v>
       </c>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
+      <c r="D19" s="39"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="39"/>
     </row>
     <row r="20" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="28" t="s">
@@ -8083,10 +8083,10 @@
       <c r="C20" s="41" t="s">
         <v>604</v>
       </c>
-      <c r="D20" s="34"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="34"/>
-      <c r="G20" s="34"/>
+      <c r="D20" s="39"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="39"/>
     </row>
     <row r="21" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="28" t="s">
@@ -8099,13 +8099,13 @@
       <c r="C21" s="41" t="s">
         <v>606</v>
       </c>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
+      <c r="D21" s="39"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
     </row>
     <row r="23" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="31" t="s">
+      <c r="A23" s="40" t="s">
         <v>607</v>
       </c>
       <c r="B23" s="32"/>
@@ -8116,7 +8116,7 @@
       <c r="G23" s="32"/>
     </row>
     <row r="24" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="31" t="s">
+      <c r="A24" s="40" t="s">
         <v>608</v>
       </c>
       <c r="B24" s="32"/>
@@ -8127,7 +8127,7 @@
       <c r="G24" s="32"/>
     </row>
     <row r="25" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="31" t="s">
+      <c r="A25" s="40" t="s">
         <v>609</v>
       </c>
       <c r="B25" s="32"/>
@@ -8169,7 +8169,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="31" t="s">
         <v>610</v>
       </c>
       <c r="B1" s="32"/>
@@ -8179,7 +8179,7 @@
       <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="34" t="s">
         <v>611</v>
       </c>
       <c r="B2" s="32"/>
@@ -8413,7 +8413,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="31" t="s">
         <v>663</v>
       </c>
       <c r="B1" s="32"/>
@@ -8423,7 +8423,7 @@
       <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="34" t="s">
         <v>664</v>
       </c>
       <c r="B2" s="32"/>
@@ -10123,7 +10123,7 @@
       <c r="F89" s="32"/>
     </row>
     <row r="90" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="31" t="s">
+      <c r="A90" s="40" t="s">
         <v>905</v>
       </c>
       <c r="B90" s="32"/>
@@ -10133,7 +10133,7 @@
       <c r="F90" s="32"/>
     </row>
     <row r="91" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="31" t="s">
+      <c r="A91" s="40" t="s">
         <v>906</v>
       </c>
       <c r="B91" s="32"/>
@@ -10143,7 +10143,7 @@
       <c r="F91" s="32"/>
     </row>
     <row r="92" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="31" t="s">
+      <c r="A92" s="40" t="s">
         <v>907</v>
       </c>
       <c r="B92" s="32"/>
@@ -10153,7 +10153,7 @@
       <c r="F92" s="32"/>
     </row>
     <row r="93" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="31" t="s">
+      <c r="A93" s="40" t="s">
         <v>908</v>
       </c>
       <c r="B93" s="32"/>
@@ -10192,7 +10192,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="31" t="s">
         <v>909</v>
       </c>
       <c r="B1" s="32"/>
@@ -10200,7 +10200,7 @@
       <c r="D1" s="32"/>
     </row>
     <row r="2" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="34" t="s">
         <v>910</v>
       </c>
       <c r="B2" s="32"/>
@@ -10329,7 +10329,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="31" t="s">
         <v>938</v>
       </c>
       <c r="B1" s="32"/>
@@ -10338,7 +10338,7 @@
       <c r="E1" s="32"/>
     </row>
     <row r="2" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="34" t="s">
         <v>939</v>
       </c>
       <c r="B2" s="32"/>

</xml_diff>

<commit_message>
3. günün görevleri bitti
</commit_message>
<xml_diff>
--- a/docs/Kalori_Sayaci_20_Gunluk_Staj_Plani.xlsx
+++ b/docs/Kalori_Sayaci_20_Gunluk_Staj_Plani.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekin\Desktop\FDN\kalori\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD612BF1-F48D-4EDF-9429-19A8502C7F82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E35E02A-AD78-4C12-8DE7-4988D4271986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3284,15 +3284,15 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3743,169 +3743,169 @@
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
     </row>
     <row r="6" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="39"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="39"/>
-      <c r="F6" s="39"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="38"/>
     </row>
     <row r="7" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="38"/>
     </row>
     <row r="8" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="38"/>
     </row>
     <row r="9" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="38"/>
     </row>
     <row r="10" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="38" t="s">
+      <c r="B10" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="38"/>
     </row>
     <row r="11" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="38" t="s">
+      <c r="B11" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="38"/>
+      <c r="F11" s="38"/>
     </row>
     <row r="12" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="38" t="s">
+      <c r="B12" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="38"/>
     </row>
     <row r="13" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="38" t="s">
+      <c r="B13" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="38"/>
     </row>
     <row r="14" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="38" t="s">
+      <c r="B14" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="39"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="38"/>
     </row>
     <row r="15" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="38" t="s">
+      <c r="B15" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="39"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="38"/>
     </row>
     <row r="16" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="38"/>
     </row>
     <row r="17" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="38" t="s">
+      <c r="B17" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="38"/>
     </row>
     <row r="18" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="38" t="s">
+      <c r="B18" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="38"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
@@ -3946,11 +3946,11 @@
       </c>
       <c r="D22" s="6">
         <f>SUMIFS('Sprint Plani'!$H$4:$H$77,'Sprint Plani'!$A$4:$A$77,$A22,'Sprint Plani'!$K$4:$K$77,"Tamamlandı")</f>
-        <v>23.5</v>
+        <v>26</v>
       </c>
       <c r="E22" s="7">
         <f>IFERROR($D22/$C22,0)</f>
-        <v>0.55952380952380953</v>
+        <v>0.61904761904761907</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>39</v>
@@ -4042,11 +4042,11 @@
       </c>
       <c r="D26" s="10">
         <f>SUM(D22:D25)</f>
-        <v>23.5</v>
+        <v>26</v>
       </c>
       <c r="E26" s="11">
         <f>IFERROR(D26/C26,0)</f>
-        <v>0.14114114114114115</v>
+        <v>0.15615615615615616</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>47</v>
@@ -4084,11 +4084,11 @@
       </c>
       <c r="C30" s="14">
         <f>COUNTIF('Sprint Plani'!$K$4:$K$77,$B30)</f>
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D30" s="15">
         <f>SUMIF('Sprint Plani'!$K$4:$K$77,$B30,'Sprint Plani'!$H$4:$H$77)</f>
-        <v>143</v>
+        <v>140.5</v>
       </c>
       <c r="E30" s="14"/>
       <c r="F30" s="16" t="s">
@@ -4124,11 +4124,11 @@
       </c>
       <c r="C32" s="14">
         <f>COUNTIF('Sprint Plani'!$K$4:$K$77,$B32)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D32" s="15">
         <f>SUMIF('Sprint Plani'!$K$4:$K$77,$B32,'Sprint Plani'!$H$4:$H$77)</f>
-        <v>23.5</v>
+        <v>26</v>
       </c>
       <c r="E32" s="14"/>
       <c r="F32" s="16" t="s">
@@ -4241,7 +4241,7 @@
       </c>
     </row>
     <row r="40" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="40" t="s">
+      <c r="A40" s="39" t="s">
         <v>73</v>
       </c>
       <c r="B40" s="32"/>
@@ -4251,7 +4251,7 @@
       <c r="F40" s="32"/>
     </row>
     <row r="41" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="40" t="s">
+      <c r="A41" s="39" t="s">
         <v>74</v>
       </c>
       <c r="B41" s="32"/>
@@ -4261,7 +4261,7 @@
       <c r="F41" s="32"/>
     </row>
     <row r="42" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="40" t="s">
+      <c r="A42" s="39" t="s">
         <v>75</v>
       </c>
       <c r="B42" s="32"/>
@@ -4271,7 +4271,7 @@
       <c r="F42" s="32"/>
     </row>
     <row r="43" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="40" t="s">
+      <c r="A43" s="39" t="s">
         <v>76</v>
       </c>
       <c r="B43" s="32"/>
@@ -4281,7 +4281,7 @@
       <c r="F43" s="32"/>
     </row>
     <row r="44" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="40" t="s">
+      <c r="A44" s="39" t="s">
         <v>77</v>
       </c>
       <c r="B44" s="32"/>
@@ -4296,7 +4296,7 @@
       </c>
     </row>
     <row r="47" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="37" t="s">
+      <c r="A47" s="40" t="s">
         <v>79</v>
       </c>
       <c r="B47" s="32"/>
@@ -4306,7 +4306,7 @@
       <c r="F47" s="32"/>
     </row>
     <row r="48" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="37" t="s">
+      <c r="A48" s="40" t="s">
         <v>80</v>
       </c>
       <c r="B48" s="32"/>
@@ -4316,7 +4316,7 @@
       <c r="F48" s="32"/>
     </row>
     <row r="49" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="37" t="s">
+      <c r="A49" s="40" t="s">
         <v>81</v>
       </c>
       <c r="B49" s="32"/>
@@ -4326,7 +4326,7 @@
       <c r="F49" s="32"/>
     </row>
     <row r="50" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="37" t="s">
+      <c r="A50" s="40" t="s">
         <v>82</v>
       </c>
       <c r="B50" s="32"/>
@@ -4336,7 +4336,7 @@
       <c r="F50" s="32"/>
     </row>
     <row r="51" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="37" t="s">
+      <c r="A51" s="40" t="s">
         <v>83</v>
       </c>
       <c r="B51" s="32"/>
@@ -4347,17 +4347,6 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B9:F9"/>
     <mergeCell ref="A41:F41"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B16:F16"/>
@@ -4373,6 +4362,17 @@
     <mergeCell ref="A49:F49"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="A40:F40"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B9:F9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4880,7 +4880,7 @@
         <v>143</v>
       </c>
       <c r="K15" s="19" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="92.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -8067,10 +8067,10 @@
       <c r="C19" s="41" t="s">
         <v>602</v>
       </c>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="39"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="38"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="38"/>
     </row>
     <row r="20" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="28" t="s">
@@ -8083,10 +8083,10 @@
       <c r="C20" s="41" t="s">
         <v>604</v>
       </c>
-      <c r="D20" s="39"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="39"/>
-      <c r="G20" s="39"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="38"/>
+      <c r="F20" s="38"/>
+      <c r="G20" s="38"/>
     </row>
     <row r="21" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="28" t="s">
@@ -8099,13 +8099,13 @@
       <c r="C21" s="41" t="s">
         <v>606</v>
       </c>
-      <c r="D21" s="39"/>
-      <c r="E21" s="39"/>
-      <c r="F21" s="39"/>
-      <c r="G21" s="39"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
+      <c r="F21" s="38"/>
+      <c r="G21" s="38"/>
     </row>
     <row r="23" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="40" t="s">
+      <c r="A23" s="39" t="s">
         <v>607</v>
       </c>
       <c r="B23" s="32"/>
@@ -8116,7 +8116,7 @@
       <c r="G23" s="32"/>
     </row>
     <row r="24" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="40" t="s">
+      <c r="A24" s="39" t="s">
         <v>608</v>
       </c>
       <c r="B24" s="32"/>
@@ -8127,7 +8127,7 @@
       <c r="G24" s="32"/>
     </row>
     <row r="25" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="40" t="s">
+      <c r="A25" s="39" t="s">
         <v>609</v>
       </c>
       <c r="B25" s="32"/>
@@ -10123,7 +10123,7 @@
       <c r="F89" s="32"/>
     </row>
     <row r="90" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="40" t="s">
+      <c r="A90" s="39" t="s">
         <v>905</v>
       </c>
       <c r="B90" s="32"/>
@@ -10133,7 +10133,7 @@
       <c r="F90" s="32"/>
     </row>
     <row r="91" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="40" t="s">
+      <c r="A91" s="39" t="s">
         <v>906</v>
       </c>
       <c r="B91" s="32"/>
@@ -10143,7 +10143,7 @@
       <c r="F91" s="32"/>
     </row>
     <row r="92" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="40" t="s">
+      <c r="A92" s="39" t="s">
         <v>907</v>
       </c>
       <c r="B92" s="32"/>
@@ -10153,7 +10153,7 @@
       <c r="F92" s="32"/>
     </row>
     <row r="93" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="40" t="s">
+      <c r="A93" s="39" t="s">
         <v>908</v>
       </c>
       <c r="B93" s="32"/>

</xml_diff>

<commit_message>
feat(db): swipe oturumları, geri bildiirim sebepleri ve deste filtreleri
</commit_message>
<xml_diff>
--- a/docs/Kalori_Sayaci_20_Gunluk_Staj_Plani.xlsx
+++ b/docs/Kalori_Sayaci_20_Gunluk_Staj_Plani.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekin\Desktop\FDN\kalori\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E35E02A-AD78-4C12-8DE7-4988D4271986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F30C482D-1E04-4C78-A174-8C550CACE4D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="288" windowWidth="23232" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ozet Dashboard" sheetId="1" r:id="rId1"/>
@@ -3284,13 +3284,13 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3743,169 +3743,169 @@
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="38"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
     </row>
     <row r="6" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="38"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="39"/>
     </row>
     <row r="7" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="37" t="s">
+      <c r="B7" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="38"/>
-      <c r="D7" s="38"/>
-      <c r="E7" s="38"/>
-      <c r="F7" s="38"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
     </row>
     <row r="8" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="37" t="s">
+      <c r="B8" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="38"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="38"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
     </row>
     <row r="9" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="37" t="s">
+      <c r="B9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="38"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="38"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
     </row>
     <row r="10" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="38"/>
-      <c r="D10" s="38"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="38"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
     </row>
     <row r="11" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="37" t="s">
+      <c r="B11" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="38"/>
-      <c r="D11" s="38"/>
-      <c r="E11" s="38"/>
-      <c r="F11" s="38"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
     </row>
     <row r="12" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="37" t="s">
+      <c r="B12" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="38"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="38"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="39"/>
     </row>
     <row r="13" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="37" t="s">
+      <c r="B13" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="38"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
     </row>
     <row r="14" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="37" t="s">
+      <c r="B14" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="38"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="39"/>
     </row>
     <row r="15" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="37" t="s">
+      <c r="B15" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="38"/>
-      <c r="D15" s="38"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="38"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="39"/>
     </row>
     <row r="16" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="37" t="s">
+      <c r="B16" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="38"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="38"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="39"/>
+      <c r="F16" s="39"/>
     </row>
     <row r="17" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="37" t="s">
+      <c r="B17" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="38"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="39"/>
+      <c r="F17" s="39"/>
     </row>
     <row r="18" spans="1:6" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="37" t="s">
+      <c r="B18" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="38"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="39"/>
+      <c r="F18" s="39"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
@@ -3946,11 +3946,11 @@
       </c>
       <c r="D22" s="6">
         <f>SUMIFS('Sprint Plani'!$H$4:$H$77,'Sprint Plani'!$A$4:$A$77,$A22,'Sprint Plani'!$K$4:$K$77,"Tamamlandı")</f>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E22" s="7">
         <f>IFERROR($D22/$C22,0)</f>
-        <v>0.61904761904761907</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>39</v>
@@ -4042,11 +4042,11 @@
       </c>
       <c r="D26" s="10">
         <f>SUM(D22:D25)</f>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E26" s="11">
         <f>IFERROR(D26/C26,0)</f>
-        <v>0.15615615615615616</v>
+        <v>0.16816816816816818</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>47</v>
@@ -4084,11 +4084,11 @@
       </c>
       <c r="C30" s="14">
         <f>COUNTIF('Sprint Plani'!$K$4:$K$77,$B30)</f>
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D30" s="15">
         <f>SUMIF('Sprint Plani'!$K$4:$K$77,$B30,'Sprint Plani'!$H$4:$H$77)</f>
-        <v>140.5</v>
+        <v>138.5</v>
       </c>
       <c r="E30" s="14"/>
       <c r="F30" s="16" t="s">
@@ -4124,11 +4124,11 @@
       </c>
       <c r="C32" s="14">
         <f>COUNTIF('Sprint Plani'!$K$4:$K$77,$B32)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D32" s="15">
         <f>SUMIF('Sprint Plani'!$K$4:$K$77,$B32,'Sprint Plani'!$H$4:$H$77)</f>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E32" s="14"/>
       <c r="F32" s="16" t="s">
@@ -4241,7 +4241,7 @@
       </c>
     </row>
     <row r="40" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="39" t="s">
+      <c r="A40" s="37" t="s">
         <v>73</v>
       </c>
       <c r="B40" s="32"/>
@@ -4251,7 +4251,7 @@
       <c r="F40" s="32"/>
     </row>
     <row r="41" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="39" t="s">
+      <c r="A41" s="37" t="s">
         <v>74</v>
       </c>
       <c r="B41" s="32"/>
@@ -4261,7 +4261,7 @@
       <c r="F41" s="32"/>
     </row>
     <row r="42" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="39" t="s">
+      <c r="A42" s="37" t="s">
         <v>75</v>
       </c>
       <c r="B42" s="32"/>
@@ -4271,7 +4271,7 @@
       <c r="F42" s="32"/>
     </row>
     <row r="43" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="39" t="s">
+      <c r="A43" s="37" t="s">
         <v>76</v>
       </c>
       <c r="B43" s="32"/>
@@ -4281,7 +4281,7 @@
       <c r="F43" s="32"/>
     </row>
     <row r="44" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="39" t="s">
+      <c r="A44" s="37" t="s">
         <v>77</v>
       </c>
       <c r="B44" s="32"/>
@@ -4347,6 +4347,17 @@
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B9:F9"/>
     <mergeCell ref="A41:F41"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B16:F16"/>
@@ -4362,17 +4373,6 @@
     <mergeCell ref="A49:F49"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="A40:F40"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B9:F9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4915,7 +4915,7 @@
         <v>95</v>
       </c>
       <c r="K16" s="17" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="54.45" customHeight="1" x14ac:dyDescent="0.3">
@@ -8067,10 +8067,10 @@
       <c r="C19" s="41" t="s">
         <v>602</v>
       </c>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="38"/>
-      <c r="G19" s="38"/>
+      <c r="D19" s="39"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="39"/>
     </row>
     <row r="20" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="28" t="s">
@@ -8083,10 +8083,10 @@
       <c r="C20" s="41" t="s">
         <v>604</v>
       </c>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="38"/>
-      <c r="G20" s="38"/>
+      <c r="D20" s="39"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="39"/>
     </row>
     <row r="21" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="28" t="s">
@@ -8099,13 +8099,13 @@
       <c r="C21" s="41" t="s">
         <v>606</v>
       </c>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="38"/>
+      <c r="D21" s="39"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
     </row>
     <row r="23" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="39" t="s">
+      <c r="A23" s="37" t="s">
         <v>607</v>
       </c>
       <c r="B23" s="32"/>
@@ -8116,7 +8116,7 @@
       <c r="G23" s="32"/>
     </row>
     <row r="24" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="39" t="s">
+      <c r="A24" s="37" t="s">
         <v>608</v>
       </c>
       <c r="B24" s="32"/>
@@ -8127,7 +8127,7 @@
       <c r="G24" s="32"/>
     </row>
     <row r="25" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="39" t="s">
+      <c r="A25" s="37" t="s">
         <v>609</v>
       </c>
       <c r="B25" s="32"/>
@@ -10123,7 +10123,7 @@
       <c r="F89" s="32"/>
     </row>
     <row r="90" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="39" t="s">
+      <c r="A90" s="37" t="s">
         <v>905</v>
       </c>
       <c r="B90" s="32"/>
@@ -10133,7 +10133,7 @@
       <c r="F90" s="32"/>
     </row>
     <row r="91" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="39" t="s">
+      <c r="A91" s="37" t="s">
         <v>906</v>
       </c>
       <c r="B91" s="32"/>
@@ -10143,7 +10143,7 @@
       <c r="F91" s="32"/>
     </row>
     <row r="92" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="39" t="s">
+      <c r="A92" s="37" t="s">
         <v>907</v>
       </c>
       <c r="B92" s="32"/>
@@ -10153,7 +10153,7 @@
       <c r="F92" s="32"/>
     </row>
     <row r="93" spans="1:6" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="39" t="s">
+      <c r="A93" s="37" t="s">
         <v>908</v>
       </c>
       <c r="B93" s="32"/>

</xml_diff>